<commit_message>
Track tokens, cost, timing — update config.md after run
</commit_message>
<xml_diff>
--- a/experiments/experiment_1/tracking.xlsx
+++ b/experiments/experiment_1/tracking.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I257"/>
+  <dimension ref="A1:L257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -490,6 +490,9 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -536,6 +539,21 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Turns</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens In</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens Out</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Cost ($)</t>
         </is>
       </c>
     </row>

</xml_diff>